<commit_message>
Encode filters in URL #922 in views (e.g. directory) create criteria from url and update filter components when going into case keep the criteria in the vaadin session cache add reset button do this for cases directory
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -273,7 +273,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.10.0-SNAPSHOT</t>
+    <t>1.11.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -2344,8 +2344,8 @@
       <c r="E35" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F35" s="2" t="s">
-        <v>20</v>
+      <c r="F35" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="G35" s="2" t="s">
         <v>20</v>
@@ -2512,8 +2512,8 @@
       <c r="E38" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F38" s="2" t="s">
-        <v>20</v>
+      <c r="F38" s="1" t="s">
+        <v>19</v>
       </c>
       <c r="G38" s="2" t="s">
         <v>20</v>

</xml_diff>

<commit_message>
#900 reactivated automatic generation of caption properties and fixed genColumn entries
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1316" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1388" uniqueCount="98">
   <si>
     <t>User Right</t>
   </si>
@@ -291,10 +291,22 @@
     <t>TREATMENT_DELETE</t>
   </si>
   <si>
+    <t>CLINICAL_COURSE_VIEW</t>
+  </si>
+  <si>
+    <t>CLINICAL_VISIT_CREATE</t>
+  </si>
+  <si>
+    <t>CLINICAL_VISIT_EDIT</t>
+  </si>
+  <si>
+    <t>CLINICAL_VISIT_DELETE</t>
+  </si>
+  <si>
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.12.0-SNAPSHOT</t>
+    <t>1.13.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -422,7 +434,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:S73"/>
+  <dimension ref="A1:S77"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.0" customWidth="true"/>
@@ -4533,6 +4545,230 @@
         <v>20</v>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="s" s="3">
+        <v>92</v>
+      </c>
+      <c r="B74" t="s">
+        <v>92</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I74" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O74" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P74" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="Q74" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="R74" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="s" s="3">
+        <v>93</v>
+      </c>
+      <c r="B75" t="s">
+        <v>93</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q75" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="R75" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="s" s="3">
+        <v>94</v>
+      </c>
+      <c r="B76" t="s">
+        <v>94</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D76" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q76" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="R76" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="s" s="3">
+        <v>95</v>
+      </c>
+      <c r="B77" t="s">
+        <v>95</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="M77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="N77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="O77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="P77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="Q77" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="R77" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -4545,12 +4781,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#1277 - Added content to the aggregate reports app view, added save and retrieval logic, overhauled disease configuration cache and disease configuration facade, added aggregate diseases, added caseBased property to disease
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2092" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2158" uniqueCount="123">
   <si>
     <t>User Right</t>
   </si>
@@ -369,10 +369,19 @@
     <t>POPULATION_MANAGE</t>
   </si>
   <si>
+    <t>LINE_LISTING_CONFIGURE</t>
+  </si>
+  <si>
+    <t>LINE_LISTING_CONFIGURE_NATION</t>
+  </si>
+  <si>
+    <t>AGGREGATE_REPORT_VIEW</t>
+  </si>
+  <si>
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.30.0-SNAPSHOT</t>
+    <t>1.31.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -500,7 +509,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:W95"/>
+  <dimension ref="A1:W98"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.0" customWidth="true"/>
@@ -6987,6 +6996,210 @@
         <v>24</v>
       </c>
     </row>
+    <row r="96">
+      <c r="A96" t="s" s="3">
+        <v>118</v>
+      </c>
+      <c r="B96" t="s">
+        <v>118</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D96" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E96" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U96" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="V96" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="s" s="3">
+        <v>119</v>
+      </c>
+      <c r="B97" t="s">
+        <v>119</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="J97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="R97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="S97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="T97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="U97" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="V97" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="s" s="3">
+        <v>120</v>
+      </c>
+      <c r="B98" t="s">
+        <v>120</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="E98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="I98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="K98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="M98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="N98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="O98" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="P98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="S98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="T98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="U98" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="V98" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
@@ -6999,12 +7212,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#1637: Change facility selection
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -63,7 +63,7 @@
     <t>National Observer</t>
   </si>
   <si>
-    <t>State Observer</t>
+    <t>Region Observer</t>
   </si>
   <si>
     <t>District Observer</t>
@@ -108,7 +108,7 @@
     <t>District</t>
   </si>
   <si>
-    <t>Health facility</t>
+    <t>Facility</t>
   </si>
   <si>
     <t>Community</t>
@@ -492,7 +492,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.44.0-SNAPSHOT</t>
+    <t>1.45.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
#1637: finish web part and consider facility type in imports
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3052" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3127" uniqueCount="163">
   <si>
     <t>User Right</t>
   </si>
@@ -63,7 +63,7 @@
     <t>National Observer</t>
   </si>
   <si>
-    <t>State Observer</t>
+    <t>Region Observer</t>
   </si>
   <si>
     <t>District Observer</t>
@@ -108,7 +108,7 @@
     <t>District</t>
   </si>
   <si>
-    <t>Health facility</t>
+    <t>Facility</t>
   </si>
   <si>
     <t>Community</t>
@@ -255,7 +255,7 @@
     <t>CONTACT_REASSIGN_CASE</t>
   </si>
   <si>
-    <t>CONTACT_CREATE_PIA_ACCOUNT</t>
+    <t>MANAGE_EXTERNAL_SYMPTOM_JOURNAL</t>
   </si>
   <si>
     <t>VISIT_CREATE</t>
@@ -288,6 +288,15 @@
     <t>TASK_DELETE</t>
   </si>
   <si>
+    <t>ACTION_CREATE</t>
+  </si>
+  <si>
+    <t>ACTION_DELETE</t>
+  </si>
+  <si>
+    <t>ACTION_EDIT</t>
+  </si>
+  <si>
     <t>EVENT_CREATE</t>
   </si>
   <si>
@@ -492,7 +501,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.45.0-SNAPSHOT</t>
+    <t>1.46.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -620,7 +629,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:Z122"/>
+  <dimension ref="A1:Z125"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.0" customWidth="true"/>
@@ -2073,8 +2082,8 @@
       <c r="L19" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M19" s="2" t="s">
-        <v>38</v>
+      <c r="M19" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>37</v>
@@ -2227,8 +2236,8 @@
       <c r="L21" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M21" s="2" t="s">
-        <v>38</v>
+      <c r="M21" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N21" s="1" t="s">
         <v>37</v>
@@ -2304,8 +2313,8 @@
       <c r="L22" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M22" s="2" t="s">
-        <v>38</v>
+      <c r="M22" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N22" s="2" t="s">
         <v>38</v>
@@ -2689,8 +2698,8 @@
       <c r="L27" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M27" s="2" t="s">
-        <v>38</v>
+      <c r="M27" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>37</v>
@@ -2766,8 +2775,8 @@
       <c r="L28" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M28" s="2" t="s">
-        <v>38</v>
+      <c r="M28" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N28" s="1" t="s">
         <v>37</v>
@@ -4972,35 +4981,35 @@
       <c r="C57" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M57" s="1" t="s">
-        <v>37</v>
+      <c r="D57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M57" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N57" s="2" t="s">
         <v>38</v>
@@ -5008,23 +5017,23 @@
       <c r="O57" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="T57" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="U57" s="1" t="s">
-        <v>37</v>
+      <c r="P57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T57" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U57" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="V57" s="2" t="s">
         <v>38</v>
@@ -5132,8 +5141,8 @@
       <c r="E59" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F59" s="2" t="s">
-        <v>38</v>
+      <c r="F59" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G59" s="2" t="s">
         <v>38</v>
@@ -5141,23 +5150,23 @@
       <c r="H59" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I59" s="1" t="s">
-        <v>37</v>
+      <c r="I59" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J59" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K59" s="1" t="s">
-        <v>37</v>
+      <c r="K59" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L59" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M59" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N59" s="1" t="s">
-        <v>37</v>
+      <c r="M59" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="O59" s="2" t="s">
         <v>38</v>
@@ -5171,17 +5180,17 @@
       <c r="R59" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S59" s="1" t="s">
-        <v>37</v>
+      <c r="S59" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T59" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U59" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V59" s="1" t="s">
-        <v>37</v>
+      <c r="U59" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V59" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W59" s="2" t="s">
         <v>38</v>
@@ -5203,35 +5212,35 @@
       <c r="C60" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M60" s="2" t="s">
-        <v>38</v>
+      <c r="D60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M60" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N60" s="2" t="s">
         <v>38</v>
@@ -5239,23 +5248,23 @@
       <c r="O60" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="T60" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="U60" s="2" t="s">
-        <v>38</v>
+      <c r="P60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T60" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U60" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="V60" s="2" t="s">
         <v>38</v>
@@ -5283,11 +5292,11 @@
       <c r="D61" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E61" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F61" s="2" t="s">
-        <v>38</v>
+      <c r="E61" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G61" s="2" t="s">
         <v>38</v>
@@ -5307,8 +5316,8 @@
       <c r="L61" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M61" s="2" t="s">
-        <v>38</v>
+      <c r="M61" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N61" s="2" t="s">
         <v>38</v>
@@ -5360,8 +5369,8 @@
       <c r="D62" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E62" s="2" t="s">
-        <v>38</v>
+      <c r="E62" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F62" s="2" t="s">
         <v>38</v>
@@ -5387,20 +5396,20 @@
       <c r="M62" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N62" s="2" t="s">
-        <v>38</v>
+      <c r="N62" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="O62" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P62" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q62" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R62" s="1" t="s">
-        <v>37</v>
+      <c r="P62" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q62" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R62" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="S62" s="1" t="s">
         <v>37</v>
@@ -5434,14 +5443,14 @@
       <c r="C63" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D63" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E63" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F63" s="1" t="s">
-        <v>37</v>
+      <c r="D63" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G63" s="2" t="s">
         <v>38</v>
@@ -5461,8 +5470,8 @@
       <c r="L63" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M63" s="1" t="s">
-        <v>37</v>
+      <c r="M63" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N63" s="2" t="s">
         <v>38</v>
@@ -5514,11 +5523,11 @@
       <c r="D64" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E64" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F64" s="1" t="s">
-        <v>37</v>
+      <c r="E64" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G64" s="2" t="s">
         <v>38</v>
@@ -5538,8 +5547,8 @@
       <c r="L64" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M64" s="1" t="s">
-        <v>37</v>
+      <c r="M64" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N64" s="2" t="s">
         <v>38</v>
@@ -5603,14 +5612,14 @@
       <c r="H65" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I65" s="2" t="s">
-        <v>38</v>
+      <c r="I65" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="J65" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K65" s="2" t="s">
-        <v>38</v>
+      <c r="K65" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>38</v>
@@ -5624,26 +5633,26 @@
       <c r="O65" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P65" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q65" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R65" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S65" s="2" t="s">
-        <v>38</v>
+      <c r="P65" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q65" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R65" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S65" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T65" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U65" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V65" s="2" t="s">
-        <v>38</v>
+      <c r="U65" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V65" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W65" s="2" t="s">
         <v>38</v>
@@ -5662,23 +5671,23 @@
       <c r="B66" t="s">
         <v>101</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D66" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E66" s="2" t="s">
-        <v>38</v>
+      <c r="C66" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D66" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F66" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G66" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H66" s="1" t="s">
-        <v>37</v>
+      <c r="G66" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>38</v>
@@ -5692,8 +5701,8 @@
       <c r="L66" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M66" s="2" t="s">
-        <v>38</v>
+      <c r="M66" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N66" s="2" t="s">
         <v>38</v>
@@ -5751,26 +5760,26 @@
       <c r="F67" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="G67" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H67" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I67" s="1" t="s">
-        <v>37</v>
+      <c r="G67" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I67" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J67" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K67" s="1" t="s">
-        <v>37</v>
+      <c r="K67" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L67" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M67" s="2" t="s">
-        <v>38</v>
+      <c r="M67" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N67" s="2" t="s">
         <v>38</v>
@@ -5778,17 +5787,17 @@
       <c r="O67" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P67" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q67" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R67" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S67" s="1" t="s">
-        <v>37</v>
+      <c r="P67" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q67" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R67" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S67" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T67" s="2" t="s">
         <v>38</v>
@@ -5819,8 +5828,8 @@
       <c r="C68" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D68" s="2" t="s">
-        <v>38</v>
+      <c r="D68" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>38</v>
@@ -5893,8 +5902,8 @@
       <c r="B69" t="s">
         <v>104</v>
       </c>
-      <c r="C69" s="1" t="s">
-        <v>37</v>
+      <c r="C69" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="D69" s="2" t="s">
         <v>38</v>
@@ -5902,14 +5911,14 @@
       <c r="E69" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F69" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G69" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H69" s="2" t="s">
-        <v>38</v>
+      <c r="F69" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H69" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="I69" s="2" t="s">
         <v>38</v>
@@ -5973,29 +5982,29 @@
       <c r="C70" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I70" s="2" t="s">
-        <v>38</v>
+      <c r="D70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K70" s="2" t="s">
-        <v>38</v>
+      <c r="K70" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>38</v>
@@ -6009,17 +6018,17 @@
       <c r="O70" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R70" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S70" s="2" t="s">
-        <v>38</v>
+      <c r="P70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R70" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S70" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T70" s="2" t="s">
         <v>38</v>
@@ -6050,11 +6059,11 @@
       <c r="C71" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D71" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E71" s="1" t="s">
-        <v>37</v>
+      <c r="D71" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E71" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>38</v>
@@ -6086,26 +6095,26 @@
       <c r="O71" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P71" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q71" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R71" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S71" s="1" t="s">
-        <v>37</v>
+      <c r="P71" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q71" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R71" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S71" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T71" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U71" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V71" s="1" t="s">
-        <v>37</v>
+      <c r="U71" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V71" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W71" s="2" t="s">
         <v>38</v>
@@ -6127,8 +6136,8 @@
       <c r="C72" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D72" s="1" t="s">
-        <v>37</v>
+      <c r="D72" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>38</v>
@@ -6201,14 +6210,14 @@
       <c r="B73" t="s">
         <v>108</v>
       </c>
-      <c r="C73" s="2" t="s">
-        <v>38</v>
+      <c r="C73" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="D73" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="E73" s="1" t="s">
-        <v>37</v>
+      <c r="E73" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>38</v>
@@ -6296,14 +6305,14 @@
       <c r="H74" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I74" s="1" t="s">
-        <v>37</v>
+      <c r="I74" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J74" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K74" s="1" t="s">
-        <v>37</v>
+      <c r="K74" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L74" s="2" t="s">
         <v>38</v>
@@ -6311,8 +6320,8 @@
       <c r="M74" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N74" s="1" t="s">
-        <v>37</v>
+      <c r="N74" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="O74" s="2" t="s">
         <v>38</v>
@@ -6361,8 +6370,8 @@
       <c r="D75" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E75" s="1" t="s">
-        <v>37</v>
+      <c r="E75" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>38</v>
@@ -6373,14 +6382,14 @@
       <c r="H75" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I75" s="1" t="s">
-        <v>37</v>
+      <c r="I75" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J75" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K75" s="1" t="s">
-        <v>37</v>
+      <c r="K75" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L75" s="2" t="s">
         <v>38</v>
@@ -6388,8 +6397,8 @@
       <c r="M75" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N75" s="1" t="s">
-        <v>37</v>
+      <c r="N75" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="O75" s="2" t="s">
         <v>38</v>
@@ -6403,17 +6412,17 @@
       <c r="R75" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S75" s="1" t="s">
-        <v>37</v>
+      <c r="S75" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T75" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U75" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V75" s="1" t="s">
-        <v>37</v>
+      <c r="U75" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V75" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W75" s="2" t="s">
         <v>38</v>
@@ -6432,14 +6441,14 @@
       <c r="B76" t="s">
         <v>111</v>
       </c>
-      <c r="C76" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D76" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>38</v>
+      <c r="C76" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D76" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>38</v>
@@ -6512,11 +6521,11 @@
       <c r="C77" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D77" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E77" s="2" t="s">
-        <v>38</v>
+      <c r="D77" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E77" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>38</v>
@@ -6527,14 +6536,14 @@
       <c r="H77" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I77" s="2" t="s">
-        <v>38</v>
+      <c r="I77" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="J77" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K77" s="2" t="s">
-        <v>38</v>
+      <c r="K77" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="L77" s="2" t="s">
         <v>38</v>
@@ -6542,32 +6551,32 @@
       <c r="M77" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N77" s="2" t="s">
-        <v>38</v>
+      <c r="N77" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="O77" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P77" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q77" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R77" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S77" s="2" t="s">
-        <v>38</v>
+      <c r="P77" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q77" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R77" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S77" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T77" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U77" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V77" s="2" t="s">
-        <v>38</v>
+      <c r="U77" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V77" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W77" s="2" t="s">
         <v>38</v>
@@ -6589,11 +6598,11 @@
       <c r="C78" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D78" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E78" s="2" t="s">
-        <v>38</v>
+      <c r="D78" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E78" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>38</v>
@@ -6604,14 +6613,14 @@
       <c r="H78" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I78" s="2" t="s">
-        <v>38</v>
+      <c r="I78" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="J78" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K78" s="2" t="s">
-        <v>38</v>
+      <c r="K78" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="L78" s="2" t="s">
         <v>38</v>
@@ -6619,8 +6628,8 @@
       <c r="M78" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N78" s="2" t="s">
-        <v>38</v>
+      <c r="N78" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="O78" s="2" t="s">
         <v>38</v>
@@ -6634,17 +6643,17 @@
       <c r="R78" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S78" s="2" t="s">
-        <v>38</v>
+      <c r="S78" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T78" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U78" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V78" s="2" t="s">
-        <v>38</v>
+      <c r="U78" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V78" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W78" s="2" t="s">
         <v>38</v>
@@ -6666,8 +6675,8 @@
       <c r="C79" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D79" s="2" t="s">
-        <v>38</v>
+      <c r="D79" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>38</v>
@@ -6743,11 +6752,11 @@
       <c r="C80" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D80" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E80" s="1" t="s">
-        <v>37</v>
+      <c r="D80" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E80" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>38</v>
@@ -6779,26 +6788,26 @@
       <c r="O80" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P80" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q80" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R80" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S80" s="1" t="s">
-        <v>37</v>
+      <c r="P80" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q80" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R80" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S80" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T80" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U80" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V80" s="1" t="s">
-        <v>37</v>
+      <c r="U80" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V80" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W80" s="2" t="s">
         <v>38</v>
@@ -6820,8 +6829,8 @@
       <c r="C81" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D81" s="1" t="s">
-        <v>37</v>
+      <c r="D81" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>38</v>
@@ -6856,8 +6865,8 @@
       <c r="O81" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P81" s="1" t="s">
-        <v>37</v>
+      <c r="P81" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="Q81" s="2" t="s">
         <v>38</v>
@@ -6897,11 +6906,11 @@
       <c r="C82" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D82" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E82" s="1" t="s">
-        <v>37</v>
+      <c r="D82" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E82" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>38</v>
@@ -6942,17 +6951,17 @@
       <c r="R82" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S82" s="1" t="s">
-        <v>37</v>
+      <c r="S82" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T82" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U82" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V82" s="1" t="s">
-        <v>37</v>
+      <c r="U82" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V82" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W82" s="2" t="s">
         <v>38</v>
@@ -6974,11 +6983,11 @@
       <c r="C83" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D83" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E83" s="2" t="s">
-        <v>38</v>
+      <c r="D83" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E83" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>38</v>
@@ -7010,26 +7019,26 @@
       <c r="O83" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P83" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q83" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R83" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S83" s="2" t="s">
-        <v>38</v>
+      <c r="P83" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q83" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R83" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S83" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T83" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U83" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V83" s="2" t="s">
-        <v>38</v>
+      <c r="U83" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V83" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W83" s="2" t="s">
         <v>38</v>
@@ -7087,8 +7096,8 @@
       <c r="O84" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P84" s="2" t="s">
-        <v>38</v>
+      <c r="P84" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="Q84" s="2" t="s">
         <v>38</v>
@@ -7128,11 +7137,11 @@
       <c r="C85" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D85" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E85" s="2" t="s">
-        <v>38</v>
+      <c r="D85" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E85" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>38</v>
@@ -7173,17 +7182,17 @@
       <c r="R85" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S85" s="2" t="s">
-        <v>38</v>
+      <c r="S85" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T85" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U85" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V85" s="2" t="s">
-        <v>38</v>
+      <c r="U85" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V85" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W85" s="2" t="s">
         <v>38</v>
@@ -7205,14 +7214,14 @@
       <c r="C86" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F86" s="1" t="s">
-        <v>37</v>
+      <c r="D86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F86" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G86" s="2" t="s">
         <v>38</v>
@@ -7220,47 +7229,47 @@
       <c r="H86" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N86" s="1" t="s">
-        <v>37</v>
+      <c r="I86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N86" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="O86" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S86" s="1" t="s">
-        <v>37</v>
+      <c r="P86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S86" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T86" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U86" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V86" s="1" t="s">
-        <v>37</v>
+      <c r="U86" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V86" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W86" s="2" t="s">
         <v>38</v>
@@ -7285,11 +7294,11 @@
       <c r="D87" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F87" s="1" t="s">
-        <v>37</v>
+      <c r="E87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F87" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>38</v>
@@ -7297,11 +7306,11 @@
       <c r="H87" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J87" s="1" t="s">
-        <v>37</v>
+      <c r="I87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="K87" s="2" t="s">
         <v>38</v>
@@ -7309,35 +7318,35 @@
       <c r="L87" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N87" s="1" t="s">
-        <v>37</v>
+      <c r="M87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N87" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="O87" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S87" s="1" t="s">
-        <v>37</v>
+      <c r="P87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S87" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T87" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U87" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V87" s="1" t="s">
-        <v>37</v>
+      <c r="U87" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V87" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W87" s="2" t="s">
         <v>38</v>
@@ -7359,8 +7368,8 @@
       <c r="C88" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D88" s="1" t="s">
-        <v>37</v>
+      <c r="D88" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>38</v>
@@ -7380,11 +7389,11 @@
       <c r="J88" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K88" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L88" s="1" t="s">
-        <v>37</v>
+      <c r="K88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L88" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="M88" s="2" t="s">
         <v>38</v>
@@ -7395,14 +7404,14 @@
       <c r="O88" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P88" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q88" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R88" s="1" t="s">
-        <v>37</v>
+      <c r="P88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q88" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R88" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="S88" s="2" t="s">
         <v>38</v>
@@ -7439,11 +7448,11 @@
       <c r="D89" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E89" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F89" s="2" t="s">
-        <v>38</v>
+      <c r="E89" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>38</v>
@@ -7451,23 +7460,23 @@
       <c r="H89" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I89" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J89" s="2" t="s">
-        <v>38</v>
+      <c r="I89" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J89" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K89" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L89" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M89" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N89" s="2" t="s">
-        <v>38</v>
+      <c r="L89" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M89" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N89" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="O89" s="2" t="s">
         <v>38</v>
@@ -7481,17 +7490,17 @@
       <c r="R89" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="S89" s="2" t="s">
-        <v>38</v>
+      <c r="S89" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T89" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U89" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V89" s="2" t="s">
-        <v>38</v>
+      <c r="U89" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V89" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W89" s="2" t="s">
         <v>38</v>
@@ -7513,14 +7522,14 @@
       <c r="C90" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D90" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E90" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F90" s="2" t="s">
-        <v>38</v>
+      <c r="D90" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E90" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G90" s="2" t="s">
         <v>38</v>
@@ -7540,8 +7549,8 @@
       <c r="L90" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="M90" s="2" t="s">
-        <v>38</v>
+      <c r="M90" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N90" s="1" t="s">
         <v>37</v>
@@ -7549,14 +7558,14 @@
       <c r="O90" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P90" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q90" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R90" s="2" t="s">
-        <v>38</v>
+      <c r="P90" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q90" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R90" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="S90" s="1" t="s">
         <v>37</v>
@@ -7564,11 +7573,11 @@
       <c r="T90" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U90" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V90" s="2" t="s">
-        <v>38</v>
+      <c r="U90" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V90" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W90" s="2" t="s">
         <v>38</v>
@@ -7590,8 +7599,8 @@
       <c r="C91" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D91" s="2" t="s">
-        <v>38</v>
+      <c r="D91" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>38</v>
@@ -7605,17 +7614,17 @@
       <c r="H91" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I91" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J91" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K91" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L91" s="2" t="s">
-        <v>38</v>
+      <c r="I91" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K91" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L91" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="M91" s="2" t="s">
         <v>38</v>
@@ -7626,17 +7635,17 @@
       <c r="O91" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P91" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q91" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R91" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S91" s="1" t="s">
-        <v>37</v>
+      <c r="P91" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q91" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R91" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S91" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T91" s="2" t="s">
         <v>38</v>
@@ -7667,8 +7676,8 @@
       <c r="C92" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D92" s="2" t="s">
-        <v>38</v>
+      <c r="D92" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>38</v>
@@ -7682,14 +7691,14 @@
       <c r="H92" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I92" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J92" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K92" s="2" t="s">
-        <v>38</v>
+      <c r="I92" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J92" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K92" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="L92" s="2" t="s">
         <v>38</v>
@@ -7703,17 +7712,17 @@
       <c r="O92" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P92" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q92" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R92" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S92" s="1" t="s">
-        <v>37</v>
+      <c r="P92" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q92" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R92" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S92" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T92" s="2" t="s">
         <v>38</v>
@@ -7774,8 +7783,8 @@
       <c r="M93" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="N93" s="2" t="s">
-        <v>38</v>
+      <c r="N93" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="O93" s="2" t="s">
         <v>38</v>
@@ -7839,8 +7848,8 @@
       <c r="I94" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J94" s="2" t="s">
-        <v>38</v>
+      <c r="J94" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K94" s="2" t="s">
         <v>38</v>
@@ -8301,8 +8310,8 @@
       <c r="I100" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J100" s="1" t="s">
-        <v>37</v>
+      <c r="J100" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="K100" s="2" t="s">
         <v>38</v>
@@ -8455,8 +8464,8 @@
       <c r="I102" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J102" s="2" t="s">
-        <v>38</v>
+      <c r="J102" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K102" s="2" t="s">
         <v>38</v>
@@ -8514,20 +8523,20 @@
       <c r="C103" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="H103" s="1" t="s">
-        <v>37</v>
+      <c r="D103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H103" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="I103" s="1" t="s">
         <v>37</v>
@@ -8535,41 +8544,41 @@
       <c r="J103" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="K103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="N103" s="1" t="s">
-        <v>37</v>
+      <c r="K103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N103" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="O103" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R103" s="1" t="s">
-        <v>37</v>
+      <c r="P103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R103" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="S103" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="U103" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V103" s="1" t="s">
-        <v>37</v>
+      <c r="T103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U103" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V103" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W103" s="2" t="s">
         <v>38</v>
@@ -8591,14 +8600,14 @@
       <c r="C104" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D104" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E104" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F104" s="1" t="s">
-        <v>37</v>
+      <c r="D104" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E104" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F104" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G104" s="2" t="s">
         <v>38</v>
@@ -8606,11 +8615,11 @@
       <c r="H104" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I104" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J104" s="2" t="s">
-        <v>38</v>
+      <c r="I104" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J104" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K104" s="2" t="s">
         <v>38</v>
@@ -8639,14 +8648,14 @@
       <c r="S104" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="T104" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="U104" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V104" s="1" t="s">
-        <v>37</v>
+      <c r="T104" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U104" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V104" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W104" s="2" t="s">
         <v>38</v>
@@ -8683,8 +8692,8 @@
       <c r="H105" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I105" s="2" t="s">
-        <v>38</v>
+      <c r="I105" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="J105" s="2" t="s">
         <v>38</v>
@@ -8713,8 +8722,8 @@
       <c r="R105" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S105" s="2" t="s">
-        <v>38</v>
+      <c r="S105" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T105" s="2" t="s">
         <v>38</v>
@@ -8751,56 +8760,56 @@
       <c r="E106" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="N106" s="2" t="s">
-        <v>38</v>
+      <c r="F106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="N106" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="O106" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="T106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="U106" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V106" s="2" t="s">
-        <v>38</v>
+      <c r="P106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U106" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V106" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W106" s="2" t="s">
         <v>38</v>
@@ -8825,11 +8834,11 @@
       <c r="D107" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E107" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F107" s="2" t="s">
-        <v>38</v>
+      <c r="E107" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G107" s="2" t="s">
         <v>38</v>
@@ -8867,17 +8876,17 @@
       <c r="R107" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S107" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="T107" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="U107" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V107" s="2" t="s">
-        <v>38</v>
+      <c r="S107" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="T107" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U107" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V107" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W107" s="2" t="s">
         <v>38</v>
@@ -8899,29 +8908,29 @@
       <c r="C108" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G108" s="1" t="s">
-        <v>37</v>
+      <c r="D108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G108" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="H108" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I108" s="1" t="s">
-        <v>37</v>
+      <c r="I108" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J108" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K108" s="1" t="s">
-        <v>37</v>
+      <c r="K108" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L108" s="2" t="s">
         <v>38</v>
@@ -8935,26 +8944,26 @@
       <c r="O108" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="T108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="U108" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V108" s="1" t="s">
-        <v>37</v>
+      <c r="P108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U108" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V108" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W108" s="2" t="s">
         <v>38</v>
@@ -8991,14 +9000,14 @@
       <c r="H109" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I109" s="1" t="s">
-        <v>37</v>
+      <c r="I109" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J109" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K109" s="1" t="s">
-        <v>37</v>
+      <c r="K109" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L109" s="2" t="s">
         <v>38</v>
@@ -9021,17 +9030,17 @@
       <c r="R109" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S109" s="1" t="s">
-        <v>37</v>
+      <c r="S109" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="T109" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U109" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V109" s="1" t="s">
-        <v>37</v>
+      <c r="U109" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V109" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W109" s="2" t="s">
         <v>38</v>
@@ -9056,26 +9065,26 @@
       <c r="D110" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E110" s="1" t="s">
-        <v>37</v>
+      <c r="E110" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G110" s="1" t="s">
-        <v>37</v>
+      <c r="G110" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="H110" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I110" s="1" t="s">
-        <v>37</v>
+      <c r="I110" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J110" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K110" s="1" t="s">
-        <v>37</v>
+      <c r="K110" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L110" s="2" t="s">
         <v>38</v>
@@ -9089,26 +9098,26 @@
       <c r="O110" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P110" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="Q110" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="R110" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S110" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="T110" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="U110" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="V110" s="1" t="s">
-        <v>37</v>
+      <c r="P110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U110" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V110" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="W110" s="2" t="s">
         <v>38</v>
@@ -9127,8 +9136,8 @@
       <c r="B111" t="s">
         <v>146</v>
       </c>
-      <c r="C111" s="2" t="s">
-        <v>38</v>
+      <c r="C111" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="D111" s="1" t="s">
         <v>37</v>
@@ -9142,23 +9151,23 @@
       <c r="G111" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H111" s="1" t="s">
-        <v>37</v>
+      <c r="H111" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="I111" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J111" s="1" t="s">
-        <v>37</v>
+      <c r="J111" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="K111" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L111" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M111" s="1" t="s">
-        <v>37</v>
+      <c r="L111" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M111" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N111" s="2" t="s">
         <v>38</v>
@@ -9166,17 +9175,17 @@
       <c r="O111" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P111" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q111" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R111" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S111" s="2" t="s">
-        <v>38</v>
+      <c r="P111" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q111" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R111" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S111" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T111" s="1" t="s">
         <v>37</v>
@@ -9204,14 +9213,14 @@
       <c r="B112" t="s">
         <v>147</v>
       </c>
-      <c r="C112" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="D112" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E112" s="2" t="s">
-        <v>38</v>
+      <c r="C112" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D112" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E112" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>38</v>
@@ -9222,14 +9231,14 @@
       <c r="H112" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I112" s="2" t="s">
-        <v>38</v>
+      <c r="I112" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="J112" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K112" s="2" t="s">
-        <v>38</v>
+      <c r="K112" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="L112" s="2" t="s">
         <v>38</v>
@@ -9252,17 +9261,17 @@
       <c r="R112" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="S112" s="2" t="s">
-        <v>38</v>
+      <c r="S112" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T112" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U112" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V112" s="2" t="s">
-        <v>38</v>
+      <c r="U112" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V112" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W112" s="2" t="s">
         <v>38</v>
@@ -9281,8 +9290,8 @@
       <c r="B113" t="s">
         <v>148</v>
       </c>
-      <c r="C113" s="2" t="s">
-        <v>38</v>
+      <c r="C113" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="D113" s="1" t="s">
         <v>37</v>
@@ -9290,29 +9299,29 @@
       <c r="E113" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="F113" s="1" t="s">
-        <v>37</v>
+      <c r="F113" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G113" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="H113" s="1" t="s">
-        <v>37</v>
+      <c r="H113" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="I113" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="J113" s="1" t="s">
-        <v>37</v>
+      <c r="J113" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="K113" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="L113" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M113" s="1" t="s">
-        <v>37</v>
+      <c r="L113" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M113" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N113" s="2" t="s">
         <v>38</v>
@@ -9320,17 +9329,17 @@
       <c r="O113" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="P113" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q113" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="R113" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="S113" s="2" t="s">
-        <v>38</v>
+      <c r="P113" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="Q113" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="R113" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S113" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="T113" s="1" t="s">
         <v>37</v>
@@ -9361,35 +9370,35 @@
       <c r="C114" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M114" s="2" t="s">
-        <v>38</v>
+      <c r="D114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M114" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N114" s="2" t="s">
         <v>38</v>
@@ -9409,14 +9418,14 @@
       <c r="S114" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="U114" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V114" s="2" t="s">
-        <v>38</v>
+      <c r="T114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U114" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V114" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W114" s="2" t="s">
         <v>38</v>
@@ -9435,17 +9444,17 @@
       <c r="B115" t="s">
         <v>150</v>
       </c>
-      <c r="C115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="E115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F115" s="1" t="s">
-        <v>37</v>
+      <c r="C115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F115" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G115" s="2" t="s">
         <v>38</v>
@@ -9453,20 +9462,20 @@
       <c r="H115" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L115" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M115" s="1" t="s">
-        <v>37</v>
+      <c r="I115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L115" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M115" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N115" s="2" t="s">
         <v>38</v>
@@ -9489,8 +9498,8 @@
       <c r="T115" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U115" s="1" t="s">
-        <v>37</v>
+      <c r="U115" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="V115" s="2" t="s">
         <v>38</v>
@@ -9512,38 +9521,38 @@
       <c r="B116" t="s">
         <v>151</v>
       </c>
-      <c r="C116" s="1" t="s">
-        <v>37</v>
+      <c r="C116" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="D116" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="H116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="I116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M116" s="2" t="s">
-        <v>38</v>
+      <c r="E116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="H116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="I116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M116" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N116" s="2" t="s">
         <v>38</v>
@@ -9563,14 +9572,14 @@
       <c r="S116" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="T116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="U116" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="V116" s="2" t="s">
-        <v>38</v>
+      <c r="T116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="U116" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V116" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="W116" s="2" t="s">
         <v>38</v>
@@ -9589,11 +9598,11 @@
       <c r="B117" t="s">
         <v>152</v>
       </c>
-      <c r="C117" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D117" s="1" t="s">
-        <v>37</v>
+      <c r="C117" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="D117" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>38</v>
@@ -9669,14 +9678,14 @@
       <c r="C118" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D118" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E118" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F118" s="2" t="s">
-        <v>38</v>
+      <c r="D118" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E118" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G118" s="2" t="s">
         <v>38</v>
@@ -9684,20 +9693,20 @@
       <c r="H118" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I118" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J118" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K118" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L118" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M118" s="2" t="s">
-        <v>38</v>
+      <c r="I118" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J118" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K118" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L118" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M118" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N118" s="2" t="s">
         <v>38</v>
@@ -9720,8 +9729,8 @@
       <c r="T118" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U118" s="2" t="s">
-        <v>38</v>
+      <c r="U118" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="V118" s="2" t="s">
         <v>38</v>
@@ -9749,11 +9758,11 @@
       <c r="D119" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E119" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="F119" s="1" t="s">
-        <v>37</v>
+      <c r="E119" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F119" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="G119" s="2" t="s">
         <v>38</v>
@@ -9761,20 +9770,20 @@
       <c r="H119" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I119" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J119" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="K119" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L119" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="M119" s="1" t="s">
-        <v>37</v>
+      <c r="I119" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J119" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K119" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L119" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M119" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="N119" s="2" t="s">
         <v>38</v>
@@ -9797,8 +9806,8 @@
       <c r="T119" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U119" s="1" t="s">
-        <v>37</v>
+      <c r="U119" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="V119" s="2" t="s">
         <v>38</v>
@@ -9826,8 +9835,8 @@
       <c r="D120" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E120" s="1" t="s">
-        <v>37</v>
+      <c r="E120" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="F120" s="2" t="s">
         <v>38</v>
@@ -9838,14 +9847,14 @@
       <c r="H120" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I120" s="1" t="s">
-        <v>37</v>
+      <c r="I120" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="J120" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="K120" s="1" t="s">
-        <v>37</v>
+      <c r="K120" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="L120" s="2" t="s">
         <v>38</v>
@@ -9874,8 +9883,8 @@
       <c r="T120" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U120" s="1" t="s">
-        <v>37</v>
+      <c r="U120" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="V120" s="2" t="s">
         <v>38</v>
@@ -9900,8 +9909,8 @@
       <c r="C121" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D121" s="1" t="s">
-        <v>37</v>
+      <c r="D121" s="2" t="s">
+        <v>38</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>38</v>
@@ -9977,14 +9986,14 @@
       <c r="C122" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D122" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E122" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="F122" s="2" t="s">
-        <v>38</v>
+      <c r="D122" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E122" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G122" s="2" t="s">
         <v>38</v>
@@ -9992,20 +10001,20 @@
       <c r="H122" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="I122" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="J122" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="K122" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="L122" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="M122" s="2" t="s">
-        <v>38</v>
+      <c r="I122" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J122" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="K122" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L122" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="M122" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="N122" s="2" t="s">
         <v>38</v>
@@ -10028,8 +10037,8 @@
       <c r="T122" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="U122" s="2" t="s">
-        <v>38</v>
+      <c r="U122" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="V122" s="2" t="s">
         <v>38</v>
@@ -10041,6 +10050,237 @@
         <v>38</v>
       </c>
       <c r="Y122" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="s" s="3">
+        <v>158</v>
+      </c>
+      <c r="B123" t="s">
+        <v>158</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D123" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E123" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I123" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="J123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K123" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="L123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U123" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="V123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="W123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X123" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y123" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="s" s="3">
+        <v>159</v>
+      </c>
+      <c r="B124" t="s">
+        <v>159</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D124" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="E124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="W124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X124" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y124" s="2" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="s" s="3">
+        <v>160</v>
+      </c>
+      <c r="B125" t="s">
+        <v>160</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="D125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="G125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="H125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="J125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="L125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="M125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="N125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="O125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="P125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="R125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="S125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="T125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="U125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="V125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="W125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="X125" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Y125" s="2" t="s">
         <v>38</v>
       </c>
     </row>
@@ -10056,12 +10296,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#2137 - Only display cases and contacts from the user's jurisdiction by default
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3512" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3539" uniqueCount="171">
   <si>
     <t>User Right</t>
   </si>
@@ -517,6 +517,9 @@
   </si>
   <si>
     <t>BAG_EXPORT</t>
+  </si>
+  <si>
+    <t>SORMAS_TO_SORMAS_SHARE</t>
   </si>
   <si>
     <t>SORMAS Version</t>
@@ -650,7 +653,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AB130"/>
+  <dimension ref="A1:AB131"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.0" customWidth="true"/>
@@ -1611,8 +1614,8 @@
       <c r="E12" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>40</v>
+      <c r="F12" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>40</v>
@@ -10519,8 +10522,8 @@
       <c r="N119" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="O119" s="2" t="s">
-        <v>40</v>
+      <c r="O119" s="1" t="s">
+        <v>39</v>
       </c>
       <c r="P119" s="2" t="s">
         <v>40</v>
@@ -11469,6 +11472,89 @@
         <v>40</v>
       </c>
       <c r="AA130" s="2" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="s" s="3">
+        <v>168</v>
+      </c>
+      <c r="B131" t="s">
+        <v>168</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="F131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="G131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="I131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="J131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="K131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="L131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="M131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="N131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="O131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="P131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Q131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="R131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="S131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="T131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="U131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="V131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="W131" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="X131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Y131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="Z131" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AA131" s="2" t="s">
         <v>40</v>
       </c>
     </row>
@@ -11484,12 +11570,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
#2996: Display "External ID" field for switzerland
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -525,7 +525,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.51.0-SNAPSHOT</t>
+    <t>${project.version}</t>
   </si>
 </sst>
 </file>
@@ -6926,8 +6926,8 @@
       <c r="E76" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F76" s="1" t="s">
-        <v>39</v>
+      <c r="F76" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G76" s="2" t="s">
         <v>40</v>
@@ -9825,14 +9825,14 @@
       <c r="C111" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D111" s="1" t="s">
-        <v>39</v>
+      <c r="D111" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="E111" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F111" s="1" t="s">
-        <v>39</v>
+      <c r="F111" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G111" s="2" t="s">
         <v>40</v>
@@ -9914,8 +9914,8 @@
       <c r="E112" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F112" s="1" t="s">
-        <v>39</v>
+      <c r="F112" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G112" s="2" t="s">
         <v>40</v>
@@ -11491,8 +11491,8 @@
       <c r="E131" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="F131" s="1" t="s">
-        <v>39</v>
+      <c r="F131" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="G131" s="1" t="s">
         <v>39</v>

</xml_diff>

<commit_message>
#3925 update data dictionary and user rights
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -537,7 +537,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.53.0-SNAPSHOT</t>
+    <t>1.54.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -11005,14 +11005,14 @@
       <c r="X120" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="Y120" s="2" t="s">
-        <v>41</v>
+      <c r="Y120" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="Z120" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AA120" s="2" t="s">
-        <v>41</v>
+      <c r="AA120" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="AB120" s="2" t="s">
         <v>41</v>
@@ -11091,14 +11091,14 @@
       <c r="X121" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="Y121" s="2" t="s">
-        <v>41</v>
+      <c r="Y121" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="Z121" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AA121" s="2" t="s">
-        <v>41</v>
+      <c r="AA121" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="AB121" s="2" t="s">
         <v>41</v>
@@ -11177,14 +11177,14 @@
       <c r="X122" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="Y122" s="2" t="s">
-        <v>41</v>
+      <c r="Y122" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="Z122" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AA122" s="2" t="s">
-        <v>41</v>
+      <c r="AA122" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="AB122" s="2" t="s">
         <v>41</v>
@@ -11263,14 +11263,14 @@
       <c r="X123" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="Y123" s="2" t="s">
-        <v>41</v>
+      <c r="Y123" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="Z123" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AA123" s="2" t="s">
-        <v>41</v>
+      <c r="AA123" s="1" t="s">
+        <v>40</v>
       </c>
       <c r="AB123" s="2" t="s">
         <v>41</v>
@@ -11372,8 +11372,8 @@
       <c r="C125" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D125" s="1" t="s">
-        <v>40</v>
+      <c r="D125" s="2" t="s">
+        <v>41</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>41</v>

</xml_diff>

<commit_message>
detect charset for import (#4050)
</commit_message>
<xml_diff>
--- a/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
+++ b/sormas-api/src/main/resources/doc/SORMAS_User_Rights.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4033" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4062" uniqueCount="182">
   <si>
     <t>User Right</t>
   </si>
@@ -330,6 +330,9 @@
     <t>EVENT_EDIT</t>
   </si>
   <si>
+    <t>EVENT_IMPORT</t>
+  </si>
+  <si>
     <t>EVENT_EXPORT</t>
   </si>
   <si>
@@ -555,7 +558,7 @@
     <t>SORMAS Version</t>
   </si>
   <si>
-    <t>1.57.0-SNAPSHOT</t>
+    <t>1.58.0-SNAPSHOT</t>
   </si>
 </sst>
 </file>
@@ -683,7 +686,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AD139"/>
+  <dimension ref="A1:AD140"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="35.0" customWidth="true"/>
@@ -6512,14 +6515,14 @@
       <c r="C66" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D66" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E66" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F66" s="1" t="s">
-        <v>41</v>
+      <c r="D66" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G66" s="2" t="s">
         <v>42</v>
@@ -6533,14 +6536,14 @@
       <c r="J66" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K66" s="1" t="s">
-        <v>41</v>
+      <c r="K66" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M66" s="1" t="s">
-        <v>41</v>
+      <c r="M66" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="N66" s="2" t="s">
         <v>42</v>
@@ -6548,8 +6551,8 @@
       <c r="O66" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="P66" s="1" t="s">
-        <v>41</v>
+      <c r="P66" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Q66" s="2" t="s">
         <v>42</v>
@@ -6563,20 +6566,20 @@
       <c r="T66" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U66" s="1" t="s">
-        <v>41</v>
+      <c r="U66" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V66" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W66" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X66" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="Y66" s="2" t="s">
-        <v>42</v>
+      <c r="W66" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X66" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y66" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Z66" s="2" t="s">
         <v>42</v>
@@ -6601,14 +6604,14 @@
       <c r="C67" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D67" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E67" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F67" s="2" t="s">
-        <v>42</v>
+      <c r="D67" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G67" s="2" t="s">
         <v>42</v>
@@ -6622,14 +6625,14 @@
       <c r="J67" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K67" s="2" t="s">
-        <v>42</v>
+      <c r="K67" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="L67" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M67" s="2" t="s">
-        <v>42</v>
+      <c r="M67" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="N67" s="2" t="s">
         <v>42</v>
@@ -6637,8 +6640,8 @@
       <c r="O67" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="P67" s="2" t="s">
-        <v>42</v>
+      <c r="P67" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q67" s="2" t="s">
         <v>42</v>
@@ -6652,17 +6655,17 @@
       <c r="T67" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U67" s="2" t="s">
-        <v>42</v>
+      <c r="U67" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V67" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W67" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X67" s="2" t="s">
-        <v>42</v>
+      <c r="W67" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X67" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y67" s="2" t="s">
         <v>42</v>
@@ -6690,8 +6693,8 @@
       <c r="C68" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D68" s="1" t="s">
-        <v>41</v>
+      <c r="D68" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>42</v>
@@ -6800,14 +6803,14 @@
       <c r="J69" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K69" s="1" t="s">
-        <v>41</v>
+      <c r="K69" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="L69" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M69" s="1" t="s">
-        <v>41</v>
+      <c r="M69" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="N69" s="2" t="s">
         <v>42</v>
@@ -6821,26 +6824,26 @@
       <c r="Q69" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R69" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S69" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T69" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U69" s="1" t="s">
-        <v>41</v>
+      <c r="R69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U69" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V69" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W69" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X69" s="1" t="s">
-        <v>41</v>
+      <c r="W69" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X69" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y69" s="2" t="s">
         <v>42</v>
@@ -6871,38 +6874,38 @@
       <c r="D70" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E70" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F70" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G70" s="1" t="s">
-        <v>41</v>
+      <c r="E70" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F70" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H70" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I70" s="1" t="s">
-        <v>41</v>
+      <c r="I70" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J70" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K70" s="2" t="s">
-        <v>42</v>
+      <c r="K70" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M70" s="2" t="s">
-        <v>42</v>
+      <c r="M70" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="N70" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="O70" s="1" t="s">
-        <v>41</v>
+      <c r="O70" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P70" s="2" t="s">
         <v>42</v>
@@ -6910,26 +6913,26 @@
       <c r="Q70" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R70" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S70" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T70" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U70" s="2" t="s">
-        <v>42</v>
+      <c r="R70" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S70" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T70" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U70" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V70" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W70" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X70" s="2" t="s">
-        <v>42</v>
+      <c r="W70" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X70" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y70" s="2" t="s">
         <v>42</v>
@@ -7049,20 +7052,20 @@
       <c r="D72" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E72" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F72" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G72" s="2" t="s">
-        <v>42</v>
+      <c r="E72" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G72" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H72" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I72" s="2" t="s">
-        <v>42</v>
+      <c r="I72" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J72" s="2" t="s">
         <v>42</v>
@@ -7079,8 +7082,8 @@
       <c r="N72" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="O72" s="2" t="s">
-        <v>42</v>
+      <c r="O72" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="P72" s="2" t="s">
         <v>42</v>
@@ -7138,20 +7141,20 @@
       <c r="D73" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E73" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F73" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G73" s="1" t="s">
-        <v>41</v>
+      <c r="E73" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H73" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I73" s="1" t="s">
-        <v>41</v>
+      <c r="I73" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J73" s="2" t="s">
         <v>42</v>
@@ -7168,8 +7171,8 @@
       <c r="N73" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="O73" s="1" t="s">
-        <v>41</v>
+      <c r="O73" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P73" s="2" t="s">
         <v>42</v>
@@ -7198,8 +7201,8 @@
       <c r="X73" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="Y73" s="1" t="s">
-        <v>41</v>
+      <c r="Y73" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Z73" s="2" t="s">
         <v>42</v>
@@ -7221,29 +7224,29 @@
       <c r="B74" t="s">
         <v>113</v>
       </c>
-      <c r="C74" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D74" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E74" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F74" s="2" t="s">
-        <v>42</v>
+      <c r="C74" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D74" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E74" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G74" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H74" s="1" t="s">
-        <v>41</v>
+      <c r="H74" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="I74" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J74" s="1" t="s">
-        <v>41</v>
+      <c r="J74" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="K74" s="2" t="s">
         <v>42</v>
@@ -7257,8 +7260,8 @@
       <c r="N74" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="O74" s="2" t="s">
-        <v>42</v>
+      <c r="O74" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="P74" s="2" t="s">
         <v>42</v>
@@ -7287,8 +7290,8 @@
       <c r="X74" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="Y74" s="2" t="s">
-        <v>42</v>
+      <c r="Y74" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Z74" s="2" t="s">
         <v>42</v>
@@ -7310,17 +7313,17 @@
       <c r="B75" t="s">
         <v>114</v>
       </c>
-      <c r="C75" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D75" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E75" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F75" s="1" t="s">
-        <v>41</v>
+      <c r="C75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G75" s="1" t="s">
         <v>41</v>
@@ -7334,14 +7337,14 @@
       <c r="J75" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="K75" s="1" t="s">
-        <v>41</v>
+      <c r="K75" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="L75" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M75" s="1" t="s">
-        <v>41</v>
+      <c r="M75" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="N75" s="2" t="s">
         <v>42</v>
@@ -7355,17 +7358,17 @@
       <c r="Q75" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R75" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S75" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T75" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U75" s="1" t="s">
-        <v>41</v>
+      <c r="R75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T75" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U75" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V75" s="2" t="s">
         <v>42</v>
@@ -7402,35 +7405,35 @@
       <c r="C76" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K76" s="2" t="s">
-        <v>42</v>
+      <c r="D76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K76" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="L76" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M76" s="2" t="s">
-        <v>42</v>
+      <c r="M76" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="N76" s="2" t="s">
         <v>42</v>
@@ -7444,17 +7447,17 @@
       <c r="Q76" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T76" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U76" s="2" t="s">
-        <v>42</v>
+      <c r="R76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T76" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U76" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V76" s="2" t="s">
         <v>42</v>
@@ -7669,14 +7672,14 @@
       <c r="C79" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F79" s="1" t="s">
-        <v>41</v>
+      <c r="D79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F79" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G79" s="2" t="s">
         <v>42</v>
@@ -7711,26 +7714,26 @@
       <c r="Q79" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U79" s="1" t="s">
-        <v>41</v>
+      <c r="R79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U79" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V79" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W79" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X79" s="1" t="s">
-        <v>41</v>
+      <c r="W79" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X79" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y79" s="2" t="s">
         <v>42</v>
@@ -7761,11 +7764,11 @@
       <c r="D80" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E80" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F80" s="2" t="s">
-        <v>42</v>
+      <c r="E80" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G80" s="2" t="s">
         <v>42</v>
@@ -7800,26 +7803,26 @@
       <c r="Q80" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R80" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S80" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T80" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U80" s="2" t="s">
-        <v>42</v>
+      <c r="R80" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S80" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T80" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U80" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V80" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W80" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X80" s="2" t="s">
-        <v>42</v>
+      <c r="W80" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X80" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y80" s="2" t="s">
         <v>42</v>
@@ -7844,17 +7847,17 @@
       <c r="B81" t="s">
         <v>120</v>
       </c>
-      <c r="C81" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D81" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E81" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F81" s="1" t="s">
-        <v>41</v>
+      <c r="C81" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E81" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F81" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G81" s="2" t="s">
         <v>42</v>
@@ -7933,17 +7936,17 @@
       <c r="B82" t="s">
         <v>121</v>
       </c>
-      <c r="C82" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E82" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F82" s="2" t="s">
-        <v>42</v>
+      <c r="C82" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D82" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E82" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G82" s="2" t="s">
         <v>42</v>
@@ -8028,11 +8031,11 @@
       <c r="D83" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E83" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F83" s="1" t="s">
-        <v>41</v>
+      <c r="E83" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F83" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G83" s="2" t="s">
         <v>42</v>
@@ -8046,14 +8049,14 @@
       <c r="J83" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K83" s="1" t="s">
-        <v>41</v>
+      <c r="K83" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="L83" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M83" s="1" t="s">
-        <v>41</v>
+      <c r="M83" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="N83" s="2" t="s">
         <v>42</v>
@@ -8061,32 +8064,32 @@
       <c r="O83" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="P83" s="1" t="s">
-        <v>41</v>
+      <c r="P83" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Q83" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R83" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S83" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T83" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U83" s="1" t="s">
-        <v>41</v>
+      <c r="R83" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S83" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T83" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U83" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V83" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W83" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X83" s="1" t="s">
-        <v>41</v>
+      <c r="W83" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X83" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y83" s="2" t="s">
         <v>42</v>
@@ -8156,14 +8159,14 @@
       <c r="Q84" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R84" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S84" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T84" s="2" t="s">
-        <v>42</v>
+      <c r="R84" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S84" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T84" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="U84" s="1" t="s">
         <v>41</v>
@@ -8206,11 +8209,11 @@
       <c r="D85" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E85" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F85" s="2" t="s">
-        <v>42</v>
+      <c r="E85" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G85" s="2" t="s">
         <v>42</v>
@@ -8224,14 +8227,14 @@
       <c r="J85" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K85" s="2" t="s">
-        <v>42</v>
+      <c r="K85" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="L85" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M85" s="2" t="s">
-        <v>42</v>
+      <c r="M85" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="N85" s="2" t="s">
         <v>42</v>
@@ -8239,8 +8242,8 @@
       <c r="O85" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="P85" s="2" t="s">
-        <v>42</v>
+      <c r="P85" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q85" s="2" t="s">
         <v>42</v>
@@ -8254,17 +8257,17 @@
       <c r="T85" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U85" s="2" t="s">
-        <v>42</v>
+      <c r="U85" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V85" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W85" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X85" s="2" t="s">
-        <v>42</v>
+      <c r="W85" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X85" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y85" s="2" t="s">
         <v>42</v>
@@ -8292,8 +8295,8 @@
       <c r="C86" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D86" s="2" t="s">
-        <v>42</v>
+      <c r="D86" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>42</v>
@@ -8381,14 +8384,14 @@
       <c r="C87" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D87" s="1" t="s">
-        <v>41</v>
+      <c r="D87" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F87" s="1" t="s">
-        <v>41</v>
+      <c r="F87" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G87" s="2" t="s">
         <v>42</v>
@@ -8470,8 +8473,8 @@
       <c r="C88" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D88" s="2" t="s">
-        <v>42</v>
+      <c r="D88" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>42</v>
@@ -8565,8 +8568,8 @@
       <c r="E89" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F89" s="2" t="s">
-        <v>42</v>
+      <c r="F89" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G89" s="2" t="s">
         <v>42</v>
@@ -8737,14 +8740,14 @@
       <c r="C91" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D91" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E91" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F91" s="1" t="s">
-        <v>41</v>
+      <c r="D91" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E91" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F91" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G91" s="2" t="s">
         <v>42</v>
@@ -8779,26 +8782,26 @@
       <c r="Q91" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R91" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S91" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T91" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U91" s="1" t="s">
-        <v>41</v>
+      <c r="R91" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S91" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T91" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U91" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V91" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W91" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X91" s="1" t="s">
-        <v>41</v>
+      <c r="W91" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X91" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y91" s="2" t="s">
         <v>42</v>
@@ -8829,11 +8832,11 @@
       <c r="D92" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E92" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F92" s="2" t="s">
-        <v>42</v>
+      <c r="E92" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G92" s="2" t="s">
         <v>42</v>
@@ -8871,23 +8874,23 @@
       <c r="R92" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="S92" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T92" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U92" s="2" t="s">
-        <v>42</v>
+      <c r="S92" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T92" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U92" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V92" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W92" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X92" s="2" t="s">
-        <v>42</v>
+      <c r="W92" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X92" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y92" s="2" t="s">
         <v>42</v>
@@ -8918,11 +8921,11 @@
       <c r="D93" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E93" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F93" s="1" t="s">
-        <v>41</v>
+      <c r="E93" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F93" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G93" s="2" t="s">
         <v>42</v>
@@ -8957,8 +8960,8 @@
       <c r="Q93" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R93" s="2" t="s">
-        <v>42</v>
+      <c r="R93" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="S93" s="2" t="s">
         <v>42</v>
@@ -8966,17 +8969,17 @@
       <c r="T93" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U93" s="1" t="s">
-        <v>41</v>
+      <c r="U93" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V93" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W93" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X93" s="1" t="s">
-        <v>41</v>
+      <c r="W93" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X93" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y93" s="2" t="s">
         <v>42</v>
@@ -9004,14 +9007,14 @@
       <c r="C94" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D94" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E94" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F94" s="2" t="s">
-        <v>42</v>
+      <c r="D94" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E94" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G94" s="2" t="s">
         <v>42</v>
@@ -9055,17 +9058,17 @@
       <c r="T94" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U94" s="2" t="s">
-        <v>42</v>
+      <c r="U94" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V94" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W94" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X94" s="2" t="s">
-        <v>42</v>
+      <c r="W94" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X94" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y94" s="2" t="s">
         <v>42</v>
@@ -9093,8 +9096,8 @@
       <c r="C95" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D95" s="1" t="s">
-        <v>41</v>
+      <c r="D95" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>42</v>
@@ -9182,8 +9185,8 @@
       <c r="C96" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D96" s="2" t="s">
-        <v>42</v>
+      <c r="D96" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>42</v>
@@ -9271,32 +9274,32 @@
       <c r="C97" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G97" s="1" t="s">
-        <v>41</v>
+      <c r="D97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G97" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H97" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I97" s="1" t="s">
-        <v>41</v>
+      <c r="I97" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J97" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L97" s="1" t="s">
-        <v>41</v>
+      <c r="K97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L97" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="M97" s="2" t="s">
         <v>42</v>
@@ -9304,35 +9307,35 @@
       <c r="N97" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="O97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="P97" s="1" t="s">
-        <v>41</v>
+      <c r="O97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P97" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Q97" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U97" s="1" t="s">
-        <v>41</v>
+      <c r="R97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U97" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V97" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W97" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X97" s="1" t="s">
-        <v>41</v>
+      <c r="W97" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X97" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y97" s="2" t="s">
         <v>42</v>
@@ -9363,14 +9366,14 @@
       <c r="D98" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G98" s="2" t="s">
-        <v>42</v>
+      <c r="E98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G98" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H98" s="2" t="s">
         <v>42</v>
@@ -9381,23 +9384,23 @@
       <c r="J98" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M98" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N98" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P98" s="2" t="s">
-        <v>42</v>
+      <c r="K98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M98" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N98" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P98" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q98" s="2" t="s">
         <v>42</v>
@@ -9411,17 +9414,17 @@
       <c r="T98" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="U98" s="2" t="s">
-        <v>42</v>
+      <c r="U98" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V98" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W98" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X98" s="2" t="s">
-        <v>42</v>
+      <c r="W98" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X98" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y98" s="2" t="s">
         <v>42</v>
@@ -9464,8 +9467,8 @@
       <c r="H99" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I99" s="2" t="s">
-        <v>42</v>
+      <c r="I99" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J99" s="2" t="s">
         <v>42</v>
@@ -9479,8 +9482,8 @@
       <c r="M99" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N99" s="2" t="s">
-        <v>42</v>
+      <c r="N99" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="O99" s="2" t="s">
         <v>42</v>
@@ -9541,38 +9544,38 @@
       <c r="D100" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E100" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F100" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G100" s="1" t="s">
-        <v>41</v>
+      <c r="E100" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F100" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H100" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I100" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J100" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="K100" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L100" s="1" t="s">
-        <v>41</v>
+      <c r="I100" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K100" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L100" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="M100" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N100" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O100" s="1" t="s">
-        <v>41</v>
+      <c r="N100" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O100" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P100" s="2" t="s">
         <v>42</v>
@@ -9580,14 +9583,14 @@
       <c r="Q100" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R100" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S100" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T100" s="2" t="s">
-        <v>42</v>
+      <c r="R100" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S100" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T100" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="U100" s="2" t="s">
         <v>42</v>
@@ -9595,8 +9598,8 @@
       <c r="V100" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W100" s="1" t="s">
-        <v>41</v>
+      <c r="W100" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="X100" s="2" t="s">
         <v>42</v>
@@ -9627,26 +9630,26 @@
       <c r="C101" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G101" s="2" t="s">
-        <v>42</v>
+      <c r="D101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G101" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H101" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J101" s="2" t="s">
-        <v>42</v>
+      <c r="I101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="K101" s="1" t="s">
         <v>41</v>
@@ -9654,17 +9657,17 @@
       <c r="L101" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="M101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O101" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P101" s="1" t="s">
-        <v>41</v>
+      <c r="M101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O101" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P101" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Q101" s="2" t="s">
         <v>42</v>
@@ -9678,14 +9681,14 @@
       <c r="T101" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U101" s="1" t="s">
-        <v>41</v>
+      <c r="U101" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V101" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W101" s="2" t="s">
-        <v>42</v>
+      <c r="W101" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="X101" s="2" t="s">
         <v>42</v>
@@ -9752,8 +9755,8 @@
       <c r="O102" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="P102" s="2" t="s">
-        <v>42</v>
+      <c r="P102" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q102" s="2" t="s">
         <v>42</v>
@@ -10007,8 +10010,8 @@
       <c r="K105" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L105" s="2" t="s">
-        <v>42</v>
+      <c r="L105" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="M105" s="2" t="s">
         <v>42</v>
@@ -10096,8 +10099,8 @@
       <c r="K106" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L106" s="1" t="s">
-        <v>41</v>
+      <c r="L106" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="M106" s="2" t="s">
         <v>42</v>
@@ -10274,8 +10277,8 @@
       <c r="K108" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L108" s="2" t="s">
-        <v>42</v>
+      <c r="L108" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="M108" s="2" t="s">
         <v>42</v>
@@ -10363,8 +10366,8 @@
       <c r="K109" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L109" s="1" t="s">
-        <v>41</v>
+      <c r="L109" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="M109" s="2" t="s">
         <v>42</v>
@@ -10719,8 +10722,8 @@
       <c r="K113" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L113" s="2" t="s">
-        <v>42</v>
+      <c r="L113" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="M113" s="2" t="s">
         <v>42</v>
@@ -10784,68 +10787,68 @@
       <c r="C114" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J114" s="1" t="s">
-        <v>41</v>
+      <c r="D114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J114" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="K114" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="P114" s="1" t="s">
-        <v>41</v>
+      <c r="L114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P114" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Q114" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T114" s="1" t="s">
-        <v>41</v>
+      <c r="R114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T114" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="U114" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="V114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W114" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X114" s="1" t="s">
-        <v>41</v>
+      <c r="V114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W114" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X114" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y114" s="2" t="s">
         <v>42</v>
@@ -10885,44 +10888,44 @@
       <c r="G115" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="H115" s="2" t="s">
-        <v>42</v>
+      <c r="H115" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="I115" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="J115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P115" s="2" t="s">
-        <v>42</v>
+      <c r="J115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P115" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q115" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S115" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T115" s="2" t="s">
-        <v>42</v>
+      <c r="R115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S115" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T115" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="U115" s="1" t="s">
         <v>41</v>
@@ -10962,23 +10965,23 @@
       <c r="C116" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D116" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E116" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F116" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G116" s="2" t="s">
-        <v>42</v>
+      <c r="D116" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E116" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G116" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H116" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I116" s="2" t="s">
-        <v>42</v>
+      <c r="I116" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J116" s="2" t="s">
         <v>42</v>
@@ -11013,17 +11016,17 @@
       <c r="T116" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="U116" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V116" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="W116" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X116" s="2" t="s">
-        <v>42</v>
+      <c r="U116" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V116" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W116" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X116" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y116" s="2" t="s">
         <v>42</v>
@@ -11137,17 +11140,17 @@
       <c r="B118" t="s">
         <v>157</v>
       </c>
-      <c r="C118" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D118" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E118" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F118" s="1" t="s">
-        <v>41</v>
+      <c r="C118" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F118" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G118" s="2" t="s">
         <v>42</v>
@@ -11155,23 +11158,23 @@
       <c r="H118" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I118" s="1" t="s">
-        <v>41</v>
+      <c r="I118" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J118" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K118" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L118" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M118" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N118" s="1" t="s">
-        <v>41</v>
+      <c r="K118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M118" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N118" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="O118" s="2" t="s">
         <v>42</v>
@@ -11226,8 +11229,8 @@
       <c r="B119" t="s">
         <v>158</v>
       </c>
-      <c r="C119" s="1" t="s">
-        <v>41</v>
+      <c r="C119" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="D119" s="1" t="s">
         <v>41</v>
@@ -11244,23 +11247,23 @@
       <c r="H119" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I119" s="2" t="s">
-        <v>42</v>
+      <c r="I119" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J119" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K119" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L119" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M119" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N119" s="2" t="s">
-        <v>42</v>
+      <c r="K119" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L119" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M119" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N119" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="O119" s="2" t="s">
         <v>42</v>
@@ -11321,11 +11324,11 @@
       <c r="D120" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E120" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F120" s="2" t="s">
-        <v>42</v>
+      <c r="E120" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G120" s="2" t="s">
         <v>42</v>
@@ -11410,32 +11413,32 @@
       <c r="D121" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I121" s="1" t="s">
-        <v>41</v>
+      <c r="E121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I121" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J121" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K121" s="1" t="s">
-        <v>41</v>
+      <c r="K121" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="L121" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M121" s="1" t="s">
-        <v>41</v>
+      <c r="M121" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="N121" s="2" t="s">
         <v>42</v>
@@ -11449,26 +11452,26 @@
       <c r="Q121" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="V121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W121" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X121" s="1" t="s">
-        <v>41</v>
+      <c r="R121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="V121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W121" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X121" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y121" s="2" t="s">
         <v>42</v>
@@ -11505,14 +11508,14 @@
       <c r="F122" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G122" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H122" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I122" s="2" t="s">
-        <v>42</v>
+      <c r="G122" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H122" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I122" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J122" s="2" t="s">
         <v>42</v>
@@ -11538,20 +11541,20 @@
       <c r="Q122" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R122" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S122" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T122" s="2" t="s">
-        <v>42</v>
+      <c r="R122" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S122" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T122" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="U122" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="V122" s="2" t="s">
-        <v>42</v>
+      <c r="V122" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="W122" s="1" t="s">
         <v>41</v>
@@ -11597,8 +11600,8 @@
       <c r="G123" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="H123" s="1" t="s">
-        <v>41</v>
+      <c r="H123" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="I123" s="2" t="s">
         <v>42</v>
@@ -11627,20 +11630,20 @@
       <c r="Q123" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R123" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S123" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T123" s="1" t="s">
-        <v>41</v>
+      <c r="R123" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S123" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T123" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="U123" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="V123" s="1" t="s">
-        <v>41</v>
+      <c r="V123" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="W123" s="1" t="s">
         <v>41</v>
@@ -11671,8 +11674,8 @@
       <c r="B124" t="s">
         <v>163</v>
       </c>
-      <c r="C124" s="2" t="s">
-        <v>42</v>
+      <c r="C124" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="D124" s="1" t="s">
         <v>41</v>
@@ -11683,32 +11686,32 @@
       <c r="F124" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G124" s="1" t="s">
-        <v>41</v>
+      <c r="G124" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H124" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="I124" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J124" s="1" t="s">
-        <v>41</v>
+      <c r="I124" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J124" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="K124" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L124" s="1" t="s">
-        <v>41</v>
+      <c r="L124" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="M124" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N124" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O124" s="1" t="s">
-        <v>41</v>
+      <c r="N124" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O124" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P124" s="2" t="s">
         <v>42</v>
@@ -11716,17 +11719,17 @@
       <c r="Q124" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R124" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S124" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T124" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U124" s="2" t="s">
-        <v>42</v>
+      <c r="R124" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S124" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T124" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U124" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V124" s="1" t="s">
         <v>41</v>
@@ -11740,14 +11743,14 @@
       <c r="Y124" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="Z124" s="1" t="s">
-        <v>41</v>
+      <c r="Z124" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="AA124" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AB124" s="1" t="s">
-        <v>41</v>
+      <c r="AB124" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="AC124" s="2" t="s">
         <v>42</v>
@@ -11763,41 +11766,41 @@
       <c r="C125" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O125" s="2" t="s">
-        <v>42</v>
+      <c r="D125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O125" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="P125" s="2" t="s">
         <v>42</v>
@@ -11817,14 +11820,14 @@
       <c r="U125" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="V125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="W125" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X125" s="2" t="s">
-        <v>42</v>
+      <c r="V125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W125" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X125" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y125" s="2" t="s">
         <v>42</v>
@@ -11852,44 +11855,44 @@
       <c r="C126" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="H126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="I126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="K126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="P126" s="1" t="s">
-        <v>41</v>
+      <c r="D126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P126" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Q126" s="2" t="s">
         <v>42</v>
@@ -11906,14 +11909,14 @@
       <c r="U126" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="V126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="W126" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X126" s="1" t="s">
-        <v>41</v>
+      <c r="V126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W126" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X126" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y126" s="2" t="s">
         <v>42</v>
@@ -11941,44 +11944,44 @@
       <c r="C127" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="H127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="I127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="J127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="K127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="P127" s="2" t="s">
-        <v>42</v>
+      <c r="D127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="I127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="K127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="P127" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Q127" s="2" t="s">
         <v>42</v>
@@ -11995,14 +11998,14 @@
       <c r="U127" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="V127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="W127" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X127" s="2" t="s">
-        <v>42</v>
+      <c r="V127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="W127" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X127" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y127" s="2" t="s">
         <v>42</v>
@@ -12027,44 +12030,44 @@
       <c r="B128" t="s">
         <v>167</v>
       </c>
-      <c r="C128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G128" s="1" t="s">
-        <v>41</v>
+      <c r="C128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G128" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H128" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I128" s="1" t="s">
-        <v>41</v>
+      <c r="I128" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J128" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N128" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O128" s="1" t="s">
-        <v>41</v>
+      <c r="K128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N128" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O128" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P128" s="2" t="s">
         <v>42</v>
@@ -12087,8 +12090,8 @@
       <c r="V128" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W128" s="1" t="s">
-        <v>41</v>
+      <c r="W128" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="X128" s="2" t="s">
         <v>42</v>
@@ -12096,14 +12099,14 @@
       <c r="Y128" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="Z128" s="2" t="s">
-        <v>42</v>
+      <c r="Z128" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="AA128" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AB128" s="2" t="s">
-        <v>42</v>
+      <c r="AB128" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="AC128" s="2" t="s">
         <v>42</v>
@@ -12119,41 +12122,41 @@
       <c r="C129" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G129" s="2" t="s">
-        <v>42</v>
+      <c r="D129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G129" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H129" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I129" s="2" t="s">
-        <v>42</v>
+      <c r="I129" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J129" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N129" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O129" s="2" t="s">
-        <v>42</v>
+      <c r="K129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N129" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O129" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="P129" s="2" t="s">
         <v>42</v>
@@ -12176,8 +12179,8 @@
       <c r="V129" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W129" s="2" t="s">
-        <v>42</v>
+      <c r="W129" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="X129" s="2" t="s">
         <v>42</v>
@@ -12208,8 +12211,8 @@
       <c r="C130" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D130" s="1" t="s">
-        <v>41</v>
+      <c r="D130" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="E130" s="2" t="s">
         <v>42</v>
@@ -12297,8 +12300,8 @@
       <c r="C131" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D131" s="2" t="s">
-        <v>42</v>
+      <c r="D131" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>42</v>
@@ -12386,41 +12389,41 @@
       <c r="C132" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G132" s="1" t="s">
-        <v>41</v>
+      <c r="D132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G132" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H132" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I132" s="1" t="s">
-        <v>41</v>
+      <c r="I132" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J132" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N132" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O132" s="1" t="s">
-        <v>41</v>
+      <c r="K132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N132" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O132" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P132" s="2" t="s">
         <v>42</v>
@@ -12443,8 +12446,8 @@
       <c r="V132" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W132" s="1" t="s">
-        <v>41</v>
+      <c r="W132" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="X132" s="2" t="s">
         <v>42</v>
@@ -12484,14 +12487,14 @@
       <c r="F133" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G133" s="2" t="s">
-        <v>42</v>
+      <c r="G133" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H133" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I133" s="2" t="s">
-        <v>42</v>
+      <c r="I133" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J133" s="2" t="s">
         <v>42</v>
@@ -12499,17 +12502,17 @@
       <c r="K133" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="L133" s="2" t="s">
-        <v>42</v>
+      <c r="L133" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="M133" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="N133" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O133" s="2" t="s">
-        <v>42</v>
+      <c r="N133" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O133" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="P133" s="2" t="s">
         <v>42</v>
@@ -12567,11 +12570,11 @@
       <c r="D134" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E134" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F134" s="2" t="s">
-        <v>42</v>
+      <c r="E134" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G134" s="2" t="s">
         <v>42</v>
@@ -12585,14 +12588,14 @@
       <c r="J134" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K134" s="2" t="s">
-        <v>42</v>
+      <c r="K134" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="L134" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M134" s="2" t="s">
-        <v>42</v>
+      <c r="M134" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="N134" s="2" t="s">
         <v>42</v>
@@ -12621,8 +12624,8 @@
       <c r="V134" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W134" s="2" t="s">
-        <v>42</v>
+      <c r="W134" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="X134" s="2" t="s">
         <v>42</v>
@@ -12653,8 +12656,8 @@
       <c r="C135" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D135" s="2" t="s">
-        <v>42</v>
+      <c r="D135" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="E135" s="2" t="s">
         <v>42</v>
@@ -12742,14 +12745,14 @@
       <c r="C136" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D136" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E136" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F136" s="1" t="s">
-        <v>41</v>
+      <c r="D136" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E136" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F136" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="G136" s="2" t="s">
         <v>42</v>
@@ -12763,14 +12766,14 @@
       <c r="J136" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K136" s="1" t="s">
-        <v>41</v>
+      <c r="K136" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="L136" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M136" s="1" t="s">
-        <v>41</v>
+      <c r="M136" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="N136" s="2" t="s">
         <v>42</v>
@@ -12799,8 +12802,8 @@
       <c r="V136" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W136" s="1" t="s">
-        <v>41</v>
+      <c r="W136" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="X136" s="2" t="s">
         <v>42</v>
@@ -12828,17 +12831,17 @@
       <c r="B137" t="s">
         <v>176</v>
       </c>
-      <c r="C137" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D137" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="E137" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="F137" s="2" t="s">
-        <v>42</v>
+      <c r="C137" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D137" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E137" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="G137" s="2" t="s">
         <v>42</v>
@@ -12852,14 +12855,14 @@
       <c r="J137" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K137" s="2" t="s">
-        <v>42</v>
+      <c r="K137" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="L137" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="M137" s="2" t="s">
-        <v>42</v>
+      <c r="M137" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="N137" s="2" t="s">
         <v>42</v>
@@ -12888,8 +12891,8 @@
       <c r="V137" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W137" s="2" t="s">
-        <v>42</v>
+      <c r="W137" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="X137" s="2" t="s">
         <v>42</v>
@@ -12906,8 +12909,8 @@
       <c r="AB137" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AC137" s="1" t="s">
-        <v>41</v>
+      <c r="AC137" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="138">
@@ -12917,44 +12920,44 @@
       <c r="B138" t="s">
         <v>177</v>
       </c>
-      <c r="C138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="F138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="G138" s="1" t="s">
-        <v>41</v>
+      <c r="C138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="E138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G138" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="H138" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I138" s="1" t="s">
-        <v>41</v>
+      <c r="I138" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="J138" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="M138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="N138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="O138" s="1" t="s">
-        <v>41</v>
+      <c r="K138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O138" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="P138" s="2" t="s">
         <v>42</v>
@@ -12962,26 +12965,26 @@
       <c r="Q138" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="S138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="T138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="U138" s="1" t="s">
-        <v>41</v>
+      <c r="R138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U138" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="V138" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W138" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="X138" s="1" t="s">
-        <v>41</v>
+      <c r="W138" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X138" s="2" t="s">
+        <v>42</v>
       </c>
       <c r="Y138" s="2" t="s">
         <v>42</v>
@@ -12995,8 +12998,8 @@
       <c r="AB138" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="AC138" s="2" t="s">
-        <v>42</v>
+      <c r="AC138" s="1" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="139">
@@ -13006,8 +13009,8 @@
       <c r="B139" t="s">
         <v>178</v>
       </c>
-      <c r="C139" s="2" t="s">
-        <v>42</v>
+      <c r="C139" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="D139" s="1" t="s">
         <v>41</v>
@@ -13015,35 +13018,35 @@
       <c r="E139" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="G139" s="2" t="s">
-        <v>42</v>
+      <c r="F139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="G139" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="H139" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="I139" s="2" t="s">
-        <v>42</v>
+      <c r="I139" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="J139" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="L139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="M139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="N139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="O139" s="2" t="s">
-        <v>42</v>
+      <c r="K139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="L139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="O139" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="P139" s="2" t="s">
         <v>42</v>
@@ -13051,26 +13054,26 @@
       <c r="Q139" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="R139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="S139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="T139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="U139" s="2" t="s">
-        <v>42</v>
+      <c r="R139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="S139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="T139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="U139" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="V139" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="W139" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="X139" s="2" t="s">
-        <v>42</v>
+      <c r="W139" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="X139" s="1" t="s">
+        <v>41</v>
       </c>
       <c r="Y139" s="2" t="s">
         <v>42</v>
@@ -13085,6 +13088,95 @@
         <v>42</v>
       </c>
       <c r="AC139" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="s" s="3">
+        <v>179</v>
+      </c>
+      <c r="B140" t="s">
+        <v>179</v>
+      </c>
+      <c r="C140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D140" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E140" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="F140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="L140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="M140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="N140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="O140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="P140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Q140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="S140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="T140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="U140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="V140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="W140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="X140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Y140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="Z140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB140" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="AC140" s="2" t="s">
         <v>42</v>
       </c>
     </row>
@@ -13100,12 +13192,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>